<commit_message>
Ajustes do Fun Festival: texto do topo, sem a ficha, 'como prefere ser chamado' e pergunta de como o ganhador do buy-in é definido
Nova coluna definicao no fim da planilha, no n8n e no Apps Script.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018GxLikosYoxfCGMYWvqwmN
</commit_message>
<xml_diff>
--- a/cadastro-clientes/planilha-fun-festival.xlsx
+++ b/cadastro-clientes/planilha-fun-festival.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X1"/>
+  <dimension ref="A1:Y1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -452,6 +452,7 @@
     <col width="14" customWidth="1" min="22" max="22"/>
     <col width="14" customWidth="1" min="23" max="23"/>
     <col width="20" customWidth="1" min="24" max="24"/>
+    <col width="40" customWidth="1" min="25" max="25"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
@@ -573,6 +574,11 @@
       <c r="X1" s="1" t="inlineStr">
         <is>
           <t>emailEnviadoEm</t>
+        </is>
+      </c>
+      <c r="Y1" s="1" t="inlineStr">
+        <is>
+          <t>definicao</t>
         </is>
       </c>
     </row>

</xml_diff>